<commit_message>
Auto backup 2026-06-30 09:35:01
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Perth Purchasing/AR Dib Detail.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Perth Purchasing/AR Dib Detail.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Perth Purchasing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E3D8EAF-511A-4914-AEF4-348B6228179A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{693CA427-4880-40F1-8540-E135DA1AFB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AUSTRALIA" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="58">
   <si>
     <t>DATE</t>
   </si>
@@ -183,16 +183,53 @@
   </si>
   <si>
     <t>OFFICE WORKS</t>
+  </si>
+  <si>
+    <t>TASETY BURGER</t>
+  </si>
+  <si>
+    <t>JADEED AL RAYYAN</t>
+  </si>
+  <si>
+    <t>WENZHOU SUPERMARKET</t>
+  </si>
+  <si>
+    <t>KHORI SPICAL KABAB</t>
+  </si>
+  <si>
+    <t>AL MADIN</t>
+  </si>
+  <si>
+    <t>HAIMAAN MANDI</t>
+  </si>
+  <si>
+    <t>DUBAI DUTY FREE</t>
+  </si>
+  <si>
+    <t>SHAKE SHACK ALSHAYA</t>
+  </si>
+  <si>
+    <t>E&amp;DIGITAL APP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total </t>
+  </si>
+  <si>
+    <t>DUBAI ELECTRICTY</t>
+  </si>
+  <si>
+    <t>SMART DUBAI GOVEMME</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -202,6 +239,15 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -233,11 +279,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -262,9 +309,18 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="0" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Comma 2" xfId="1" xr:uid="{A945AF09-5752-44DF-A1A8-EC2B17E84A49}"/>
+    <cellStyle name="Comma 3" xfId="2" xr:uid="{5543D2C1-C976-4579-9AC5-466A4725339D}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1103,33 +1159,56 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17" customWidth="1"/>
+    <col min="2" max="2" width="23.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="23" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
+      <c r="A2" s="22">
         <v>46160</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="23">
         <v>208.85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>46178</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="23">
+        <v>280.23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="4">
+        <v>46191</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="20">
+        <v>6018</v>
       </c>
     </row>
   </sheetData>
@@ -1176,286 +1255,462 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="2" max="2" width="21.85546875" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="16"/>
+    <col min="2" max="2" width="10.85546875" customWidth="1"/>
+    <col min="3" max="3" width="21.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="17"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="17" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B2" s="2">
         <v>46157</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3">
+      <c r="D2" s="18">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B3" s="2">
         <v>46158</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="3">
+      <c r="D3" s="18">
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B4" s="2">
         <v>46158</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3">
+      <c r="D4" s="18">
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B5" s="2">
         <v>46158</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="3">
+      <c r="D5" s="18">
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B6" s="2">
         <v>46158</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3">
+      <c r="D6" s="18">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B7" s="2">
         <v>46159</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="18">
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B8" s="2">
         <v>46160</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="3">
+      <c r="D8" s="18">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B9" s="2">
         <v>46160</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="3">
+      <c r="D9" s="18">
         <v>3.5</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B10" s="2">
         <v>46161</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="3">
+      <c r="D10" s="18">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B11" s="2">
         <v>46162</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="3">
+      <c r="D11" s="18">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B12" s="2">
         <v>46162</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="3">
+      <c r="D12" s="18">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B13" s="2">
         <v>46163</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="3">
+      <c r="D13" s="18">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B14" s="2">
         <v>46163</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="3">
+      <c r="D14" s="18">
         <v>3</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="2">
         <v>46164</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="3">
+      <c r="D15" s="18">
         <v>450.45</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B16" s="2">
         <v>46164</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="3">
+      <c r="D16" s="18">
         <v>26</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B17" s="2">
         <v>46165</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="3">
+      <c r="D17" s="18">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B18" s="2">
         <v>46165</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="3">
+      <c r="D18" s="18">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+    <row r="19" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B19" s="2">
         <v>46166</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="3">
+      <c r="D19" s="18">
         <v>161.58000000000001</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+    <row r="20" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B20" s="2">
         <v>46166</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="3">
+      <c r="D20" s="18">
         <v>16.5</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+    <row r="21" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B21" s="2">
         <v>46166</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>11</v>
       </c>
-      <c r="C21" s="3">
+      <c r="D21" s="18">
         <v>41.97</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+    <row r="22" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B22" s="2">
         <v>46175</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="3">
+      <c r="D22" s="18">
         <v>20.75</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+    <row r="23" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B23" s="2">
         <v>46177</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>11</v>
       </c>
-      <c r="C23" s="3">
+      <c r="D23" s="18">
         <v>19.010000000000002</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B24" s="2">
         <v>46177</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>32</v>
       </c>
-      <c r="C24" s="3">
+      <c r="D24" s="18">
         <v>17</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+    <row r="25" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B25" s="2">
         <v>46178</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>33</v>
       </c>
-      <c r="C25" s="3">
+      <c r="D25" s="18">
         <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B26" s="4">
+        <v>46178</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="19">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B27" s="4">
+        <v>46178</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D27" s="19">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B28" s="4">
+        <v>46179</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B29" s="4">
+        <v>46179</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="19">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B30" s="4">
+        <v>46179</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D30" s="19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B31" s="4">
+        <v>46180</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D31" s="19">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="32" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B32" s="4">
+        <v>46180</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D32" s="19">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="33" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B33" s="4">
+        <v>46182</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="20">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="34" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B34" s="4">
+        <v>46182</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D34" s="19">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="35" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B35" s="4">
+        <v>46183</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D35" s="19">
+        <v>32.75</v>
+      </c>
+    </row>
+    <row r="36" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="4">
+        <v>46183</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="19">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="37" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B37" s="4">
+        <v>46192</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D37" s="19">
+        <v>450.45</v>
+      </c>
+    </row>
+    <row r="38" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B38" s="4">
+        <v>46196</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="19">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B39" s="4">
+        <v>46196</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="19">
+        <v>43.6</v>
+      </c>
+    </row>
+    <row r="40" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B40" s="4">
+        <v>46196</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D40" s="19">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="42" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="C42" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="21">
+        <f>SUM(D2:D41)</f>
+        <v>1997.0600000000002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>